<commit_message>
CSV file exports for MX 4.0.4
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
+++ b/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rod\Desktop\EPS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\bldgs\BPSfDSPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{0C71C972-6EB7-4463-8E00-9561AF9B13FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F010D94-C047-49CA-944F-5BA970BEE308}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0869BFB6-8993-46D4-92F4-176DDAC562A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32115" yWindow="1530" windowWidth="23310" windowHeight="13380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="7" r:id="rId1"/>
-    <sheet name="BPSfDSPV" sheetId="8" r:id="rId2"/>
+    <sheet name="BPSfDSPC" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -79,7 +79,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -432,18 +432,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="61.5703125" customWidth="1"/>
     <col min="5" max="5" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -451,10 +451,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -471,13 +471,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AY7"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
@@ -632,7 +632,7 @@
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:51">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -787,7 +787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:51">
+    <row r="3" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -942,7 +942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:51">
+    <row r="4" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1097,13 +1097,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:51">
+    <row r="5" spans="1:51" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
     </row>
-    <row r="6" spans="1:51">
+    <row r="6" spans="1:51" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:51">
+    <row r="7" spans="1:51" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
     </row>
   </sheetData>
@@ -1113,6 +1113,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -1256,12 +1262,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1272,13 +1272,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47C41D4B-45D5-42A0-99A4-938B3ACB2BC7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BCB5BCB-0E87-47FD-AF4C-8354FAD51360}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BCB5BCB-0E87-47FD-AF4C-8354FAD51360}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47C41D4B-45D5-42A0-99A4-938B3ACB2BC7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9661B59D-86F4-4600-BE69-F47BDA585B84}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9661B59D-86F4-4600-BE69-F47BDA585B84}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>